<commit_message>
feat: promote five-product shortcut param aliases
</commit_message>
<xml_diff>
--- a/docs/parameter-hallucination/shortcut-gap-reanalysis/agoal/agoal_cli_param_hallucination_analysis.xlsx
+++ b/docs/parameter-hallucination/shortcut-gap-reanalysis/agoal/agoal_cli_param_hallucination_analysis.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇报总览" sheetId="1" r:id="R34a79ee0623740b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数问题明细" sheetId="2" r:id="Re71fa9aa579544c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="兜底解决方案" sheetId="3" r:id="R6c6df3eee1c34bb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前无法解决" sheetId="4" r:id="Rc9e27c430d8142e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分析依据" sheetId="5" r:id="R8eafe5ad96024862"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇报总览" sheetId="1" r:id="R72a98b5082be4751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数问题明细" sheetId="2" r:id="R13172614b82247f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="兜底解决方案" sheetId="3" r:id="R5bbbdcc9222a4520"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前无法解决" sheetId="4" r:id="R74430ad8f1c946e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分析依据" sheetId="5" r:id="R5783ae486bea45b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -532,7 +532,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>冻结基线 5f906bf8b61bc54a75f6c2b46219a1deb682b600｜正式别名表未修改｜候选、报告、五页工作簿独立交付</x:v>
+        <x:v>冻结基线 f4474b57eb1db23b1638b9574be2f5dca368a360｜正式别名表未修改｜候选、报告、五页工作簿独立交付</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -762,7 +762,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>冻结基线 5f906bf8b61bc54a75f6c2b46219a1deb682b600｜逐命令核对真实 Help/Cobra、运行时 Schema、Skill 与正式别名表</x:v>
+        <x:v>冻结基线 f4474b57eb1db23b1638b9574be2f5dca368a360｜逐命令核对真实 Help/Cobra、运行时 Schema、Skill 与正式别名表</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1363,7 +1363,7 @@
         <x:v>冻结基线</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
-        <x:v>origin/main@5f906bf8b61bc54a75f6c2b46219a1deb682b600</x:v>
+        <x:v>origin/main@f4474b57eb1db23b1638b9574be2f5dca368a360</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
         <x:v>通过</x:v>

</xml_diff>